<commit_message>
updated bug upload bug
</commit_message>
<xml_diff>
--- a/server/public/templates/lipid_template.xlsx
+++ b/server/public/templates/lipid_template.xlsx
@@ -397,13 +397,18 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:J2"/>
+  <dimension ref="A1:J3"/>
   <cols>
     <col min="1" max="1" width="24.83203125" customWidth="1"/>
     <col min="2" max="2" width="20.83203125" customWidth="1"/>
-    <col min="3" max="3" width="12.83203125" customWidth="1"/>
-    <col min="4" max="4" width="12.83203125" customWidth="1"/>
-    <col min="5" max="5" width="12.83203125" customWidth="1"/>
+    <col min="3" max="3" width="15.83203125" customWidth="1"/>
+    <col min="4" max="4" width="15.83203125" customWidth="1"/>
+    <col min="5" max="5" width="15.83203125" customWidth="1"/>
+    <col min="6" max="6" width="15.83203125" customWidth="1"/>
+    <col min="7" max="7" width="15.83203125" customWidth="1"/>
+    <col min="8" max="8" width="12.83203125" customWidth="1"/>
+    <col min="9" max="9" width="20.83203125" customWidth="1"/>
+    <col min="10" max="10" width="12.83203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -470,9 +475,41 @@
         <v>600</v>
       </c>
     </row>
+    <row r="3">
+      <c r="A3" t="str">
+        <v>(24 char hex)</v>
+      </c>
+      <c r="B3" t="str">
+        <v>(Name)</v>
+      </c>
+      <c r="C3" t="str">
+        <v>(150-200 mg/dL)</v>
+      </c>
+      <c r="D3" t="str">
+        <v>(60-150 mg/dL)</v>
+      </c>
+      <c r="E3" t="str">
+        <v>(40-60 mg/dL)</v>
+      </c>
+      <c r="F3" t="str">
+        <v>(&lt;100 mg/dL)</v>
+      </c>
+      <c r="G3" t="str">
+        <v>(2-30 mg/dL)</v>
+      </c>
+      <c r="H3" t="str">
+        <v>(&lt;3.0)</v>
+      </c>
+      <c r="I3" t="str">
+        <v>(&lt;4.5)</v>
+      </c>
+      <c r="J3" t="str">
+        <v>(400-1000 mg/dL)</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:J2"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:J3"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>